<commit_message>
Seed the id registry from the full raw survey, before any attrition
You caught this: the registry was seeded AFTER the exclusions, so 62 raw weighings had
no id at all, and a label re-admitted later would have been handed a new number at the
end of the sequence instead of its own.

The id is now assigned on the raw market survey, immediately after obs_type is encoded
and BEFORE the comment merge and every exclusion. Registry: 11,495 rows, the full raw
file. The 62 excluded weighings keep their numbers.

Verified: ids unique, contiguous 1..11,495, every id in the build present in the
registry, and 62 held for rows the build drops.

excluded_standard_unit_obs.xlsx now carries id too, so a dropped weighing is
referenceable rather than describable only by its four-part key.

snap_sense_check.xlsx and weight_correction_report.csv regenerated on the stable ids.

verify_documented_claims.py 27 of 27 OK.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/master_rename_build/tables/unit_correction_review_queue.xlsx
+++ b/outputs/master_rename_build/tables/unit_correction_review_queue.xlsx
@@ -180,7 +180,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="1">
-        <v>4442</v>
+        <v>4462</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1">
@@ -214,7 +214,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="1">
-        <v>4974</v>
+        <v>5001</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1">
@@ -248,7 +248,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="1">
-        <v>4977</v>
+        <v>5004</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1">
@@ -282,7 +282,7 @@
         <v>9</v>
       </c>
       <c r="E5" s="1">
-        <v>4972</v>
+        <v>4999</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1">
@@ -316,7 +316,7 @@
         <v>8</v>
       </c>
       <c r="E6" s="1">
-        <v>4978</v>
+        <v>5005</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1">

</xml_diff>